<commit_message>
small fix to the dataset
</commit_message>
<xml_diff>
--- a/data/exp_raw/ssexp_data.xlsx
+++ b/data/exp_raw/ssexp_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vcantarella/Documents/FuhrbergerColumns/data/exp_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21342613-B21F-3849-93A3-917B6C8ADA24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E416A8C-C208-A44D-9DB4-A7E8495644DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="180" yWindow="740" windowWidth="29400" windowHeight="16680" firstSheet="2" activeTab="12" xr2:uid="{82067E57-95C1-4A4D-B858-7597035F15DE}"/>
+    <workbookView xWindow="20" yWindow="740" windowWidth="29400" windowHeight="16680" firstSheet="2" activeTab="12" xr2:uid="{82067E57-95C1-4A4D-B858-7597035F15DE}"/>
   </bookViews>
   <sheets>
     <sheet name="general_samples_p1" sheetId="1" r:id="rId1"/>
@@ -1922,9 +1922,6 @@
     <t>063-P2T70</t>
   </si>
   <si>
-    <t>064-P275</t>
-  </si>
-  <si>
     <t>065-P2T80</t>
   </si>
   <si>
@@ -2070,6 +2067,9 @@
   </si>
   <si>
     <t>028-P1T39</t>
+  </si>
+  <si>
+    <t>064-P2T75</t>
   </si>
 </sst>
 </file>
@@ -13436,7 +13436,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B29" t="s">
         <v>542</v>
@@ -13994,14 +13994,14 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>591</v>
+        <v>640</v>
       </c>
       <c r="B63" t="s">
         <v>542</v>
       </c>
       <c r="C63" t="str" cm="1">
         <f t="array" ref="C63">_xlfn.REGEXEXTRACT(A63,"(P?B?\w*\d)$",0,1)</f>
-        <v>P275</v>
+        <v>P2T75</v>
       </c>
       <c r="D63">
         <v>33.549999999999997</v>
@@ -14012,7 +14012,7 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B64" t="s">
         <v>542</v>
@@ -14030,7 +14030,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B65" t="s">
         <v>542</v>
@@ -14048,7 +14048,7 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B66" t="s">
         <v>542</v>
@@ -14066,7 +14066,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B67" t="s">
         <v>542</v>
@@ -14084,7 +14084,7 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B68" t="s">
         <v>542</v>
@@ -14102,7 +14102,7 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B69" t="s">
         <v>542</v>
@@ -14120,7 +14120,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B70" t="s">
         <v>542</v>
@@ -14138,7 +14138,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B71" t="s">
         <v>542</v>
@@ -14156,7 +14156,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B72" t="s">
         <v>542</v>
@@ -14174,7 +14174,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B73" t="s">
         <v>542</v>
@@ -14192,7 +14192,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B74" t="s">
         <v>542</v>
@@ -14210,7 +14210,7 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B75" t="s">
         <v>542</v>
@@ -14228,7 +14228,7 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B76" t="s">
         <v>542</v>
@@ -14246,7 +14246,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B77" t="s">
         <v>542</v>
@@ -14264,7 +14264,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B78" t="s">
         <v>542</v>
@@ -14282,7 +14282,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B79" t="s">
         <v>542</v>
@@ -14300,7 +14300,7 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B80" t="s">
         <v>542</v>
@@ -14318,7 +14318,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B81" t="s">
         <v>542</v>
@@ -14336,7 +14336,7 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B82" t="s">
         <v>542</v>
@@ -14354,7 +14354,7 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B83" t="s">
         <v>542</v>
@@ -14372,7 +14372,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B84" t="s">
         <v>542</v>
@@ -14390,7 +14390,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B85" t="s">
         <v>542</v>
@@ -14408,7 +14408,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B86" t="s">
         <v>542</v>
@@ -14426,7 +14426,7 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B87" t="s">
         <v>542</v>
@@ -14444,7 +14444,7 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B88" t="s">
         <v>542</v>
@@ -14462,7 +14462,7 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B89" t="s">
         <v>542</v>
@@ -14480,7 +14480,7 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B90" t="s">
         <v>542</v>
@@ -14498,7 +14498,7 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B91" t="s">
         <v>542</v>
@@ -14516,7 +14516,7 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B92" t="s">
         <v>542</v>
@@ -14534,7 +14534,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B93" t="s">
         <v>542</v>
@@ -14552,7 +14552,7 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B94" t="s">
         <v>542</v>
@@ -14570,7 +14570,7 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B95" t="s">
         <v>542</v>
@@ -14588,7 +14588,7 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B96" t="s">
         <v>542</v>
@@ -14606,7 +14606,7 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B97" t="s">
         <v>542</v>
@@ -14624,7 +14624,7 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B98" t="s">
         <v>542</v>
@@ -14642,7 +14642,7 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B99" t="s">
         <v>542</v>
@@ -14660,7 +14660,7 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B100" t="s">
         <v>542</v>
@@ -14678,7 +14678,7 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B101" t="s">
         <v>542</v>
@@ -14690,7 +14690,7 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B102" t="s">
         <v>542</v>
@@ -14708,7 +14708,7 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B103" t="s">
         <v>542</v>
@@ -14726,7 +14726,7 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B104" t="s">
         <v>542</v>
@@ -14744,7 +14744,7 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B105" t="s">
         <v>542</v>
@@ -14762,7 +14762,7 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B106" t="s">
         <v>542</v>
@@ -14780,7 +14780,7 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B107" t="s">
         <v>542</v>
@@ -14798,7 +14798,7 @@
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B108" t="s">
         <v>542</v>
@@ -14816,7 +14816,7 @@
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B109" t="s">
         <v>542</v>
@@ -14834,7 +14834,7 @@
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B110" t="s">
         <v>542</v>
@@ -14852,7 +14852,7 @@
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B111" t="s">
         <v>542</v>
@@ -17107,13 +17107,13 @@
         <f>3/62*14</f>
         <v>0.67741935483870963</v>
       </c>
-      <c r="K76" t="e">
+      <c r="K76">
         <f>VLOOKUP(A76,IC_raw!$C$2:$E$111,3,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="L76" t="e">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="L76">
         <f>VLOOKUP(A76,IC_raw!$C$2:$E$111,2,FALSE)</f>
-        <v>#N/A</v>
+        <v>33.549999999999997</v>
       </c>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.2">

</xml_diff>